<commit_message>
[wip] buff pipline 5
</commit_message>
<xml_diff>
--- a/table_config/_tables/Battle/#BuffData-增减益Buff-02.xlsx
+++ b/table_config/_tables/Battle/#BuffData-增减益Buff-02.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25420" windowHeight="13410"/>
+    <workbookView windowHeight="17800"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="25">
   <si>
     <t>##var</t>
   </si>
@@ -43,6 +43,15 @@
     <t>effects</t>
   </si>
   <si>
+    <t>start_stack</t>
+  </si>
+  <si>
+    <t>max_stack</t>
+  </si>
+  <si>
+    <t>duration</t>
+  </si>
+  <si>
     <t>parametric</t>
   </si>
   <si>
@@ -55,6 +64,9 @@
     <t>array#sep=|,string</t>
   </si>
   <si>
+    <t>float</t>
+  </si>
+  <si>
     <t>map,Battle.BuffParam,float</t>
   </si>
   <si>
@@ -64,19 +76,31 @@
     <t>唯一id</t>
   </si>
   <si>
-    <t>Buff参数</t>
-  </si>
-  <si>
-    <t>float</t>
+    <t>开始层数</t>
+  </si>
+  <si>
+    <t>最大层数</t>
+  </si>
+  <si>
+    <t>计时器</t>
+  </si>
+  <si>
+    <t>Buff参数1</t>
+  </si>
+  <si>
+    <t>Buff参数2</t>
+  </si>
+  <si>
+    <t>Buff参数3</t>
+  </si>
+  <si>
+    <t>Buff参数4</t>
   </si>
   <si>
     <t>冻伤</t>
   </si>
   <si>
-    <t>初始层数</t>
-  </si>
-  <si>
-    <t>计时</t>
+    <t>Damage</t>
   </si>
   <si>
     <t>流血</t>
@@ -696,7 +720,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -705,6 +729,9 @@
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1020,16 +1047,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="5"/>
   <cols>
     <col min="2" max="2" width="17.3636363636364" style="1"/>
     <col min="3" max="3" width="16.2727272727273" style="2"/>
     <col min="4" max="4" width="20.8181818181818" style="2" customWidth="1"/>
-    <col min="5" max="5" width="9.18181818181818" customWidth="1"/>
+    <col min="5" max="5" width="12.9090909090909" style="3" customWidth="1"/>
+    <col min="6" max="6" width="10.6363636363636" style="3" customWidth="1"/>
+    <col min="7" max="7" width="9.54545454545454" style="3" customWidth="1"/>
+    <col min="8" max="8" width="10.6363636363636" customWidth="1"/>
+    <col min="10" max="10" width="10.6363636363636" customWidth="1"/>
+    <col min="12" max="12" width="10.6363636363636" customWidth="1"/>
+    <col min="14" max="14" width="10.6363636363636" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1045,116 +1078,149 @@
       <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:15">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
+        <v>11</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:15">
       <c r="A3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:15">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" t="s">
-        <v>11</v>
+        <v>14</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="H4" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="I4" t="s">
         <v>11</v>
       </c>
       <c r="J4" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="K4" t="s">
         <v>11</v>
       </c>
       <c r="L4" t="s">
-        <v>12</v>
+        <v>20</v>
+      </c>
+      <c r="M4" t="s">
+        <v>11</v>
+      </c>
+      <c r="N4" t="s">
+        <v>21</v>
+      </c>
+      <c r="O4" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:15">
       <c r="B5" s="1">
         <v>1002000001</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5">
-        <v>2</v>
-      </c>
-      <c r="G5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5">
+        <v>22</v>
+      </c>
+      <c r="E5" s="3">
+        <v>1</v>
+      </c>
+      <c r="F5" s="3">
         <v>5</v>
       </c>
+      <c r="G5" s="3">
+        <v>10</v>
+      </c>
+      <c r="H5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I5">
+        <v>5</v>
+      </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:15">
       <c r="B6" s="1">
         <v>1002000002</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6">
+        <v>24</v>
+      </c>
+      <c r="E6" s="3">
+        <v>1</v>
+      </c>
+      <c r="F6" s="3">
         <v>5</v>
       </c>
-      <c r="G6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6">
+      <c r="G6" s="3">
+        <v>2</v>
+      </c>
+      <c r="H6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I6">
         <v>5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="E1:L1"/>
-    <mergeCell ref="E2:L2"/>
+    <mergeCell ref="H1:O1"/>
+    <mergeCell ref="H2:O2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
[wip] buff pipline 7
</commit_message>
<xml_diff>
--- a/table_config/_tables/Battle/#BuffData-增减益Buff-02.xlsx
+++ b/table_config/_tables/Battle/#BuffData-增减益Buff-02.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="17800"/>
+    <workbookView windowWidth="20790" windowHeight="9525"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1048,18 +1048,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:O6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="5"/>
   <cols>
-    <col min="2" max="2" width="17.3636363636364" style="1"/>
-    <col min="3" max="3" width="16.2727272727273" style="2"/>
-    <col min="4" max="4" width="20.8181818181818" style="2" customWidth="1"/>
-    <col min="5" max="5" width="12.9090909090909" style="3" customWidth="1"/>
-    <col min="6" max="6" width="10.6363636363636" style="3" customWidth="1"/>
-    <col min="7" max="7" width="9.54545454545454" style="3" customWidth="1"/>
-    <col min="8" max="8" width="10.6363636363636" customWidth="1"/>
-    <col min="10" max="10" width="10.6363636363636" customWidth="1"/>
-    <col min="12" max="12" width="10.6363636363636" customWidth="1"/>
-    <col min="14" max="14" width="10.6363636363636" customWidth="1"/>
+    <col min="2" max="2" width="17.3666666666667" style="1"/>
+    <col min="3" max="3" width="16.275" style="2"/>
+    <col min="4" max="4" width="20.8166666666667" style="2" customWidth="1"/>
+    <col min="5" max="5" width="12.9083333333333" style="3" customWidth="1"/>
+    <col min="6" max="6" width="10.6333333333333" style="3" customWidth="1"/>
+    <col min="7" max="7" width="9.54166666666667" style="3" customWidth="1"/>
+    <col min="8" max="8" width="10.6333333333333" customWidth="1"/>
+    <col min="10" max="10" width="10.6333333333333" customWidth="1"/>
+    <col min="12" max="12" width="10.6333333333333" customWidth="1"/>
+    <col min="14" max="14" width="10.6333333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -1232,7 +1232,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -1244,7 +1244,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>